<commit_message>
Adding KBA and option for no template
</commit_message>
<xml_diff>
--- a/AutomateSendingOutTaxReturnsV3.xlsx
+++ b/AutomateSendingOutTaxReturnsV3.xlsx
@@ -497,7 +497,7 @@
         <v>none</v>
       </c>
       <c r="I2" s="2" t="str">
-        <v>none</v>
+        <v>X</v>
       </c>
       <c r="J2" s="2" t="str">
         <v>MA-Single</v>
@@ -518,7 +518,7 @@
         <v>2022 1040 Return - JJ</v>
       </c>
       <c r="P2" s="2" t="str">
-        <v>X</v>
+        <v>none</v>
       </c>
       <c r="Q2" s="2">
         <v>2023</v>
@@ -550,7 +550,7 @@
         <v>none</v>
       </c>
       <c r="I3" s="2" t="str">
-        <v>none</v>
+        <v>X</v>
       </c>
       <c r="J3" s="2" t="str">
         <v>MA-Single</v>
@@ -571,7 +571,7 @@
         <v>2022 1040 Return - JJ</v>
       </c>
       <c r="P3" s="2" t="str">
-        <v>X</v>
+        <v>none</v>
       </c>
       <c r="Q3" s="2">
         <v>2023</v>
@@ -603,7 +603,7 @@
         <v>none</v>
       </c>
       <c r="I4" s="2" t="str">
-        <v>none</v>
+        <v>X</v>
       </c>
       <c r="J4" s="2" t="str">
         <v>MA-Single</v>
@@ -624,7 +624,7 @@
         <v>2022 1040 Return - JJ</v>
       </c>
       <c r="P4" s="2" t="str">
-        <v>X</v>
+        <v>none</v>
       </c>
       <c r="Q4" s="2">
         <v>2023</v>
@@ -720,8 +720,8 @@
       <c r="H2" s="4" t="str">
         <v>N</v>
       </c>
-      <c r="I2" s="4" t="str">
-        <v>N</v>
+      <c r="I2" s="5" t="str">
+        <v>Y</v>
       </c>
       <c r="J2" s="2" t="str">
         <v>MA-Single</v>
@@ -741,8 +741,8 @@
       <c r="O2" s="2" t="str">
         <v>2022 1040 Return - JJ</v>
       </c>
-      <c r="P2" s="5" t="str">
-        <v>Y</v>
+      <c r="P2" s="2" t="str">
+        <v>none</v>
       </c>
       <c r="Q2" s="2">
         <v>2023</v>
@@ -767,14 +767,14 @@
       <c r="F3" s="2" t="str">
         <v>Great!</v>
       </c>
-      <c r="G3" s="2" t="str">
-        <v>none</v>
-      </c>
-      <c r="H3" s="2" t="str">
-        <v>none</v>
-      </c>
-      <c r="I3" s="2" t="str">
-        <v>none</v>
+      <c r="G3" s="4" t="str">
+        <v>N</v>
+      </c>
+      <c r="H3" s="4" t="str">
+        <v>N</v>
+      </c>
+      <c r="I3" s="6" t="str">
+        <v>Y</v>
       </c>
       <c r="J3" s="2" t="str">
         <v>MA-Single</v>
@@ -794,8 +794,8 @@
       <c r="O3" s="2" t="str">
         <v>2022 1040 Return - JJ</v>
       </c>
-      <c r="P3" s="6" t="str">
-        <v>Y</v>
+      <c r="P3" s="2" t="str">
+        <v>none</v>
       </c>
       <c r="Q3" s="2">
         <v>2023</v>
@@ -826,8 +826,8 @@
       <c r="H4" s="4" t="str">
         <v>N</v>
       </c>
-      <c r="I4" s="4" t="str">
-        <v>N</v>
+      <c r="I4" s="6" t="str">
+        <v>Y</v>
       </c>
       <c r="J4" s="2" t="str">
         <v>MA-Single</v>
@@ -847,8 +847,8 @@
       <c r="O4" s="2" t="str">
         <v>2022 1040 Return - JJ</v>
       </c>
-      <c r="P4" s="6" t="str">
-        <v>Y</v>
+      <c r="P4" s="2" t="str">
+        <v>none</v>
       </c>
       <c r="Q4" s="2">
         <v>2023</v>

</xml_diff>

<commit_message>
Fixing Link Button (Hopefully)
</commit_message>
<xml_diff>
--- a/AutomateSendingOutTaxReturnsV3.xlsx
+++ b/AutomateSendingOutTaxReturnsV3.xlsx
@@ -504,7 +504,7 @@
         <v>none</v>
       </c>
       <c r="L2" s="2" t="str">
-        <v>X</v>
+        <v>none</v>
       </c>
       <c r="M2" s="2">
         <v>750</v>
@@ -519,7 +519,7 @@
         <v>2022 1040 Return - JJ</v>
       </c>
       <c r="Q2" s="2" t="str">
-        <v>X</v>
+        <v>none</v>
       </c>
       <c r="R2" s="2">
         <v>2019</v>
@@ -642,8 +642,8 @@
       <c r="P2" s="2" t="str">
         <v>2022 1040 Return - JJ</v>
       </c>
-      <c r="Q2" s="4" t="str">
-        <v>N</v>
+      <c r="Q2" s="2" t="str">
+        <v>none</v>
       </c>
       <c r="R2" s="2">
         <v>2019</v>

</xml_diff>

<commit_message>
Fixing Invoice Issue and Making Program Quicker by removing constant name checks.
</commit_message>
<xml_diff>
--- a/AutomateSendingOutTaxReturnsV3.xlsx
+++ b/AutomateSendingOutTaxReturnsV3.xlsx
@@ -24,7 +24,7 @@
       <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none">
         <bgColor/>
@@ -44,6 +44,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFF0000"/>
+        <bgColor/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00FF00"/>
         <bgColor/>
       </patternFill>
     </fill>
@@ -73,13 +79,14 @@
   <cellStyleXfs>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="1" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -486,7 +493,7 @@
         <v>none</v>
       </c>
       <c r="F2" s="2" t="str">
-        <v>none</v>
+        <v>Hello</v>
       </c>
       <c r="G2" s="2" t="str">
         <v>none</v>
@@ -495,7 +502,7 @@
         <v>none</v>
       </c>
       <c r="I2" s="2" t="str">
-        <v>none</v>
+        <v>X</v>
       </c>
       <c r="J2" s="2" t="str">
         <v>none</v>
@@ -504,7 +511,7 @@
         <v>none</v>
       </c>
       <c r="L2" s="2" t="str">
-        <v>none</v>
+        <v>X</v>
       </c>
       <c r="M2" s="2">
         <v>750</v>
@@ -609,8 +616,8 @@
       <c r="E2" s="4" t="str">
         <v>N</v>
       </c>
-      <c r="F2" s="2" t="str">
-        <v>none</v>
+      <c r="F2" s="5" t="str">
+        <v>Y</v>
       </c>
       <c r="G2" s="4" t="str">
         <v>N</v>
@@ -618,17 +625,17 @@
       <c r="H2" s="4" t="str">
         <v>N</v>
       </c>
-      <c r="I2" s="4" t="str">
+      <c r="I2" s="6" t="str">
+        <v>Y</v>
+      </c>
+      <c r="J2" s="2" t="str">
+        <v>none</v>
+      </c>
+      <c r="K2" s="4" t="str">
         <v>N</v>
       </c>
-      <c r="J2" s="2" t="str">
-        <v>none</v>
-      </c>
-      <c r="K2" s="2" t="str">
-        <v>none</v>
-      </c>
-      <c r="L2" s="4" t="str">
-        <v>N</v>
+      <c r="L2" s="6" t="str">
+        <v>Y</v>
       </c>
       <c r="M2" s="2">
         <v>750</v>
@@ -636,7 +643,7 @@
       <c r="N2" s="2" t="str">
         <v>Personal Tax Services - JJ</v>
       </c>
-      <c r="O2" s="5" t="str">
+      <c r="O2" s="6" t="str">
         <v>Y</v>
       </c>
       <c r="P2" s="2" t="str">

</xml_diff>

<commit_message>
JJ new pauses 3-29-24
</commit_message>
<xml_diff>
--- a/AutomateSendingOutTaxReturnsV3.xlsx
+++ b/AutomateSendingOutTaxReturnsV3.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27328"/>
   <workbookPr filterPrivacy="1" codeName="ThisWorkbook"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E2FC91C0-6F9C-4FA8-BF6C-505B14C2083A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C231160-67DF-4C7E-A2D3-34D6C5C95844}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ClientList" sheetId="1" r:id="rId1"/>
@@ -13,12 +13,25 @@
     <sheet name="Log" sheetId="3" r:id="rId3"/>
     <sheet name="SuccessLog" sheetId="4" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="327" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="327" uniqueCount="69">
   <si>
     <t>Number</t>
   </si>
@@ -74,30 +87,69 @@
     <t>YearToSeal</t>
   </si>
   <si>
+    <t>BJ12</t>
+  </si>
+  <si>
+    <t>Barrera, Julie</t>
+  </si>
+  <si>
+    <t>Send Out Returns, Bill, and Efile Sigs - InvoiceInTD</t>
+  </si>
+  <si>
+    <t>none</t>
+  </si>
+  <si>
+    <t>X</t>
+  </si>
+  <si>
+    <t>MA-Single-TS</t>
+  </si>
+  <si>
+    <t>Personal Tax Services - JJ</t>
+  </si>
+  <si>
+    <t>2023 1040 Return - JJ</t>
+  </si>
+  <si>
+    <t>LC7</t>
+  </si>
+  <si>
+    <t>Lesher, Christian &amp; Sara</t>
+  </si>
+  <si>
+    <t>Y</t>
+  </si>
+  <si>
+    <t>N</t>
+  </si>
+  <si>
+    <t>SF2</t>
+  </si>
+  <si>
+    <t>Finney, Stephen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Big increase in income this year compared to last! Your wages almost doubled and your withholdings kept up for the most part. You owe a little but not too much considering your overall income. We noted your $6.5k backdoor Roth IRA contribution and made sure to make it non-taxable. Finally, we also made sure to file you in 2 states - MA and RI. Everything else looked good. Please let me know if any questions – thanks. </t>
+  </si>
+  <si>
+    <t>AA1</t>
+  </si>
+  <si>
+    <t>Aiken, Kathleen &amp; Carillo, Catherine</t>
+  </si>
+  <si>
+    <t>Very similar to last year income wise in nearly all respects EXCEPT for your gambling winnings  – nice! It lowered your refund a bit but not much.  We are filing in MS due to this but you don’t owe any money to them as your income was not enough to incur taxes there.  We continue to itemize in Alabama - that added almost $1k to your refund thanks to the medical expenses.   Everything else looked good. Please let me know if any questions – thanks.</t>
+  </si>
+  <si>
     <t>BC7</t>
   </si>
   <si>
     <t>Brennan, Christopher &amp; Anne</t>
   </si>
   <si>
-    <t>Send Out Returns, Bill, and Efile Sigs - InvoiceInTD</t>
-  </si>
-  <si>
-    <t>none</t>
-  </si>
-  <si>
     <t>You owe a bit due to a BIG gain on your Vertex share sales (a good thing of course except now when you have to pay taxes on it!).  The gain is taxed at the most favorable long term capital gains rate and we adjusted your cost basis so you weren’t double taxed.  Everything else was very similar to last year.  Hope you are well - let me know if any questions - thanks!</t>
   </si>
   <si>
-    <t>X</t>
-  </si>
-  <si>
-    <t>Personal Tax Services - JJ</t>
-  </si>
-  <si>
-    <t>2023 1040 Return - JJ</t>
-  </si>
-  <si>
     <t>WM8</t>
   </si>
   <si>
@@ -107,9 +159,6 @@
     <t>Your mother had good withholdings and thus the estate is getting a great federal refund.  Additionally there is a nice MA refund as we got $887 for the MA Senior Circuit Breaker Credit.  My condolences again on your loss - let me know if any questions - thanks.</t>
   </si>
   <si>
-    <t>MA-Single-TS</t>
-  </si>
-  <si>
     <t>KS3</t>
   </si>
   <si>
@@ -146,47 +195,67 @@
     <t>You had some great interest and dividends this year and that is why you owe the slightest of amounts now.  That said it’s good to get interest!  My computer just completely crashed this week but the data was backed up - made me think of how you saved my bacon back in the day!  Hope all is well - let me know if any questions - thanks.</t>
   </si>
   <si>
-    <t>Y</t>
-  </si>
-  <si>
-    <t>N</t>
-  </si>
-  <si>
-    <t>SF2</t>
-  </si>
-  <si>
-    <t>Finney, Stephen</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Big increase in income this year compared to last! Your wages almost doubled and your withholdings kept up for the most part. You owe a little but not too much considering your overall income. We noted your $6.5k backdoor Roth IRA contribution and made sure to make it non-taxable. Finally, we also made sure to file you in 2 states - MA and RI. Everything else looked good. Please let me know if any questions – thanks. </t>
-  </si>
-  <si>
-    <t>AA1</t>
-  </si>
-  <si>
-    <t>Aiken, Kathleen &amp; Carillo, Catherine</t>
-  </si>
-  <si>
-    <t>Very similar to last year income wise in nearly all respects EXCEPT for your gambling winnings  – nice! It lowered your refund a bit but not much.  We are filing in MS due to this but you don’t owe any money to them as your income was not enough to incur taxes there.  We continue to itemize in Alabama - that added almost $1k to your refund thanks to the medical expenses.   Everything else looked good. Please let me know if any questions – thanks.</t>
-  </si>
-  <si>
-    <t>SD3</t>
-  </si>
-  <si>
-    <t>Single, Dummy</t>
+    <t>BJ13</t>
+  </si>
+  <si>
+    <t>Bonanno, Jasmine</t>
+  </si>
+  <si>
+    <t>Second verse, almost the same as the first! Very similar to last year wage income wise – you owe a little but not too much considering your overall income. Your wages went up $17k and your withholdings kept up. You didn't have a lot of capital gains ($4k) - they were all long term and we made sure to adjust the cost basis to ensure you weren’t double taxed. Finally we told you about the Roth income limit so that you took out $1,090 from it so you wouldn’t be penalized. You should be aware of this limit going forward and use the backdoor Roth method to get money into a Roth going forward. Everything else looked good. Please let me know if any questions – thanks.</t>
+  </si>
+  <si>
+    <t>CK6</t>
+  </si>
+  <si>
+    <t>Carmody, Karen</t>
+  </si>
+  <si>
+    <t>Your business swung from a loss to a nice income of $21k after taking out all possible deductions. Your new job had some nice withholdings and thus you don’t owe that much even though you had sizable business income. Everything else stayed similar to previous years. Please let me know if any questions - thanks.</t>
+  </si>
+  <si>
+    <t>GA14</t>
+  </si>
+  <si>
+    <t>Ganguly, Auroop &amp; Debashree</t>
+  </si>
+  <si>
+    <t>Similar to last year wage income wise – you owe a little but not too much considering your overall income. Your wages went up $75k and your withholdings kept up for the most part. We reported Auroop’s side income properly, including creating a Schedule E for the royalties. The new thing was Shree’s business - we added that and took all available deductions. This reduced the amount you owed in taxes by $972. Everything else looked good. Please let me know if any questions – thanks.</t>
+  </si>
+  <si>
+    <t>WA6</t>
+  </si>
+  <si>
+    <t>Walter, Johannes &amp; Sever, Sanja</t>
+  </si>
+  <si>
+    <t>Nice refund this year as you got most of your withholdings back due to slightly less income - everything was the same generally speaking as last year but just a little less business income. We took all possible tax deductions on each of your business returns, including the home office deduction. I set you up with a new Schedule E to report Sanja’s royalty income. Finally, made sure to discuss with you the tax implications of Sanja moving to Texas. All in all, a great year for you with exciting changes coming up! Let me know if any questions - thanks!</t>
+  </si>
+  <si>
+    <t>GB3</t>
+  </si>
+  <si>
+    <t>Garcia Barrantes, Pedro &amp; Betancourt, Rosanna</t>
+  </si>
+  <si>
+    <t>Fixed the Schedule B for Costa Rica - thanks!</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <name val="Calibri"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="8">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -210,21 +279,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="FFFF0000"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -232,18 +297,40 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -583,10 +670,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:R7"/>
+  <dimension ref="A1:R9"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:18" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:18" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -642,78 +729,300 @@
         <v>17</v>
       </c>
     </row>
-    <row r="2" spans="1:18" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A2">
-        <v>1</v>
-      </c>
-      <c r="B2" t="s">
-        <v>50</v>
-      </c>
-      <c r="C2" t="s">
-        <v>51</v>
-      </c>
-      <c r="D2" t="s">
+    <row r="2" spans="1:18" ht="409.6" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A2" s="5">
+        <v>1</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="C2" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="D2" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="E2" t="s">
-        <v>21</v>
-      </c>
-      <c r="F2" t="s">
-        <v>22</v>
-      </c>
-      <c r="G2" t="s">
+      <c r="E2" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="F2" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="G2" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="H2" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="I2" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="J2" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="H2" t="s">
+      <c r="K2" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="L2" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="M2" s="5">
+        <v>875</v>
+      </c>
+      <c r="N2" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="O2" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="P2" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q2" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="R2" s="5">
+        <v>2023</v>
+      </c>
+    </row>
+    <row r="3" spans="1:18" ht="409.6" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A3" s="5">
+        <v>1</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="C3" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="D3" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="E3" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="F3" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="G3" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="H3" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="I3" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="J3" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="I2" t="s">
-        <v>23</v>
-      </c>
-      <c r="J2" t="s">
-        <v>21</v>
-      </c>
-      <c r="K2" t="s">
-        <v>23</v>
-      </c>
-      <c r="L2" t="s">
-        <v>23</v>
-      </c>
-      <c r="M2">
-        <v>750</v>
-      </c>
-      <c r="N2" t="s">
+      <c r="K3" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="L3" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="M3" s="5">
+        <v>650</v>
+      </c>
+      <c r="N3" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="O2" t="s">
-        <v>23</v>
-      </c>
-      <c r="P2" t="s">
+      <c r="O3" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="P3" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="Q2" t="s">
-        <v>23</v>
-      </c>
-      <c r="R2">
+      <c r="Q3" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="R3" s="5">
         <v>2023</v>
       </c>
     </row>
-    <row r="3" spans="1:18" ht="15.5" x14ac:dyDescent="0.35"/>
-    <row r="4" spans="1:18" ht="15.5" x14ac:dyDescent="0.35"/>
-    <row r="5" spans="1:18" ht="15.5" x14ac:dyDescent="0.35"/>
-    <row r="6" spans="1:18" ht="15.5" x14ac:dyDescent="0.35"/>
+    <row r="4" spans="1:18" ht="409.6" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A4" s="5">
+        <v>1</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="C4" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="D4" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="E4" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="F4" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="G4" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="H4" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="I4" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="J4" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="K4" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="L4" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="M4" s="5">
+        <v>975</v>
+      </c>
+      <c r="N4" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="O4" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="P4" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q4" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="R4" s="5">
+        <v>2023</v>
+      </c>
+    </row>
+    <row r="5" spans="1:18" ht="409.6" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A5" s="5">
+        <v>1</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="D5" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="E5" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="F5" s="6" t="s">
+        <v>65</v>
+      </c>
+      <c r="G5" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="H5" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="I5" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="J5" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="K5" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="L5" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="M5" s="5">
+        <v>950</v>
+      </c>
+      <c r="N5" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="O5" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="P5" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q5" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="R5" s="5">
+        <v>2023</v>
+      </c>
+    </row>
+    <row r="6" spans="1:18" ht="76.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A6" s="5">
+        <v>1</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="C6" s="7" t="s">
+        <v>67</v>
+      </c>
+      <c r="D6" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="E6" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="F6" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="G6" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="H6" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="I6" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="J6" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="K6" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="L6" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="M6" s="5">
+        <v>0</v>
+      </c>
+      <c r="N6" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="O6" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="P6" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q6" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="R6" s="5">
+        <v>2023</v>
+      </c>
+    </row>
     <row r="7" spans="1:18" ht="15.5" x14ac:dyDescent="0.35"/>
+    <row r="8" spans="1:18" ht="15.5" x14ac:dyDescent="0.35"/>
+    <row r="9" spans="1:18" ht="15.5" x14ac:dyDescent="0.35"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:R1 A2 D2:R2" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:R1" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:R7"/>
+  <dimension ref="A1:R3"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:18" ht="15.5" x14ac:dyDescent="0.35">
@@ -783,46 +1092,46 @@
         <v>19</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>42</v>
+        <v>28</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>43</v>
+        <v>29</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="G2" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="H2" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="I2" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="J2" t="s">
         <v>23</v>
       </c>
-      <c r="H2" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="I2" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="J2" t="s">
-        <v>21</v>
-      </c>
       <c r="K2" s="3" t="s">
-        <v>42</v>
+        <v>28</v>
       </c>
       <c r="L2" s="3" t="s">
-        <v>42</v>
+        <v>28</v>
       </c>
       <c r="M2">
-        <v>750</v>
+        <v>875</v>
       </c>
       <c r="N2" t="s">
         <v>24</v>
       </c>
       <c r="O2" s="3" t="s">
-        <v>42</v>
+        <v>28</v>
       </c>
       <c r="P2" t="s">
         <v>25</v>
       </c>
       <c r="Q2" s="3" t="s">
-        <v>42</v>
+        <v>28</v>
       </c>
       <c r="R2">
         <v>2023</v>
@@ -839,279 +1148,56 @@
         <v>27</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="E3" s="5" t="s">
-        <v>43</v>
+        <v>28</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>29</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="G3" s="6" t="s">
-        <v>23</v>
+        <v>28</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>28</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>42</v>
+        <v>28</v>
       </c>
       <c r="I3" s="3" t="s">
-        <v>42</v>
+        <v>28</v>
       </c>
       <c r="J3" t="s">
-        <v>29</v>
+        <v>21</v>
       </c>
       <c r="K3" s="3" t="s">
-        <v>42</v>
+        <v>28</v>
       </c>
       <c r="L3" s="3" t="s">
-        <v>42</v>
+        <v>28</v>
       </c>
       <c r="M3">
-        <v>900</v>
+        <v>750</v>
       </c>
       <c r="N3" t="s">
         <v>24</v>
       </c>
       <c r="O3" s="3" t="s">
-        <v>42</v>
+        <v>28</v>
       </c>
       <c r="P3" t="s">
         <v>25</v>
       </c>
       <c r="Q3" s="3" t="s">
-        <v>42</v>
+        <v>28</v>
       </c>
       <c r="R3">
         <v>2023</v>
       </c>
     </row>
-    <row r="4" spans="1:18" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A4">
-        <v>1</v>
-      </c>
-      <c r="B4" t="s">
-        <v>30</v>
-      </c>
-      <c r="C4" t="s">
-        <v>31</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="E4" s="5" t="s">
-        <v>43</v>
-      </c>
-      <c r="F4" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="G4" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="H4" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="I4" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="J4" t="s">
-        <v>29</v>
-      </c>
-      <c r="K4" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="L4" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="M4">
-        <v>750</v>
-      </c>
-      <c r="N4" t="s">
-        <v>24</v>
-      </c>
-      <c r="O4" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="P4" t="s">
-        <v>25</v>
-      </c>
-      <c r="Q4" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="R4">
-        <v>2023</v>
-      </c>
-    </row>
-    <row r="5" spans="1:18" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A5">
-        <v>1</v>
-      </c>
-      <c r="B5" t="s">
-        <v>33</v>
-      </c>
-      <c r="C5" t="s">
-        <v>34</v>
-      </c>
-      <c r="D5" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="E5" s="5" t="s">
-        <v>43</v>
-      </c>
-      <c r="F5" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="G5" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="H5" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="I5" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="J5" t="s">
-        <v>29</v>
-      </c>
-      <c r="K5" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="L5" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="M5">
-        <v>875</v>
-      </c>
-      <c r="N5" t="s">
-        <v>24</v>
-      </c>
-      <c r="O5" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="P5" t="s">
-        <v>25</v>
-      </c>
-      <c r="Q5" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="R5">
-        <v>2023</v>
-      </c>
-    </row>
-    <row r="6" spans="1:18" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A6">
-        <v>1</v>
-      </c>
-      <c r="B6" t="s">
-        <v>36</v>
-      </c>
-      <c r="C6" t="s">
-        <v>37</v>
-      </c>
-      <c r="D6" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="E6" s="5" t="s">
-        <v>43</v>
-      </c>
-      <c r="F6" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="G6" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="H6" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="I6" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="J6" t="s">
-        <v>29</v>
-      </c>
-      <c r="K6" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="L6" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="M6">
-        <v>975</v>
-      </c>
-      <c r="N6" t="s">
-        <v>24</v>
-      </c>
-      <c r="O6" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="P6" t="s">
-        <v>25</v>
-      </c>
-      <c r="Q6" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="R6">
-        <v>2023</v>
-      </c>
-    </row>
-    <row r="7" spans="1:18" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A7">
-        <v>1</v>
-      </c>
-      <c r="B7" t="s">
-        <v>39</v>
-      </c>
-      <c r="C7" t="s">
-        <v>40</v>
-      </c>
-      <c r="D7" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="E7" s="5" t="s">
-        <v>43</v>
-      </c>
-      <c r="F7" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="G7" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="H7" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="I7" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="J7" t="s">
-        <v>29</v>
-      </c>
-      <c r="K7" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="L7" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="M7">
-        <v>475</v>
-      </c>
-      <c r="N7" t="s">
-        <v>24</v>
-      </c>
-      <c r="O7" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="P7" t="s">
-        <v>25</v>
-      </c>
-      <c r="Q7" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="R7">
-        <v>2023</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:R7" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:R3" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1182,10 +1268,10 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>44</v>
+        <v>30</v>
       </c>
       <c r="C2" t="s">
-        <v>45</v>
+        <v>31</v>
       </c>
       <c r="D2" t="s">
         <v>20</v>
@@ -1194,25 +1280,25 @@
         <v>21</v>
       </c>
       <c r="F2" t="s">
-        <v>46</v>
+        <v>32</v>
       </c>
       <c r="G2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="H2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="I2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="J2" t="s">
         <v>21</v>
       </c>
       <c r="K2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="L2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="M2">
         <v>875</v>
@@ -1221,13 +1307,13 @@
         <v>24</v>
       </c>
       <c r="O2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="P2" t="s">
         <v>25</v>
       </c>
       <c r="Q2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="R2">
         <v>2023</v>
@@ -1238,10 +1324,10 @@
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>47</v>
+        <v>33</v>
       </c>
       <c r="C3" t="s">
-        <v>48</v>
+        <v>34</v>
       </c>
       <c r="D3" t="s">
         <v>20</v>
@@ -1250,25 +1336,25 @@
         <v>21</v>
       </c>
       <c r="F3" t="s">
-        <v>49</v>
+        <v>35</v>
       </c>
       <c r="G3" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="H3" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="I3" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="J3" t="s">
         <v>21</v>
       </c>
       <c r="K3" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="L3" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="M3">
         <v>750</v>
@@ -1277,13 +1363,13 @@
         <v>24</v>
       </c>
       <c r="O3" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="P3" t="s">
         <v>25</v>
       </c>
       <c r="Q3" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="R3">
         <v>2023</v>
@@ -1294,10 +1380,10 @@
         <v>1</v>
       </c>
       <c r="B4" t="s">
-        <v>18</v>
+        <v>36</v>
       </c>
       <c r="C4" t="s">
-        <v>19</v>
+        <v>37</v>
       </c>
       <c r="D4" t="s">
         <v>20</v>
@@ -1306,25 +1392,25 @@
         <v>21</v>
       </c>
       <c r="F4" t="s">
-        <v>22</v>
+        <v>38</v>
       </c>
       <c r="G4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="H4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="I4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="J4" t="s">
         <v>21</v>
       </c>
       <c r="K4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="L4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="M4">
         <v>750</v>
@@ -1333,13 +1419,13 @@
         <v>24</v>
       </c>
       <c r="O4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="P4" t="s">
         <v>25</v>
       </c>
       <c r="Q4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="R4">
         <v>2023</v>
@@ -1350,10 +1436,10 @@
         <v>1</v>
       </c>
       <c r="B5" t="s">
-        <v>26</v>
+        <v>39</v>
       </c>
       <c r="C5" t="s">
-        <v>27</v>
+        <v>40</v>
       </c>
       <c r="D5" t="s">
         <v>20</v>
@@ -1362,25 +1448,25 @@
         <v>21</v>
       </c>
       <c r="F5" t="s">
-        <v>28</v>
+        <v>41</v>
       </c>
       <c r="G5" t="s">
+        <v>22</v>
+      </c>
+      <c r="H5" t="s">
+        <v>22</v>
+      </c>
+      <c r="I5" t="s">
+        <v>22</v>
+      </c>
+      <c r="J5" t="s">
         <v>23</v>
       </c>
-      <c r="H5" t="s">
-        <v>23</v>
-      </c>
-      <c r="I5" t="s">
-        <v>23</v>
-      </c>
-      <c r="J5" t="s">
-        <v>29</v>
-      </c>
       <c r="K5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="L5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="M5">
         <v>900</v>
@@ -1389,13 +1475,13 @@
         <v>24</v>
       </c>
       <c r="O5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="P5" t="s">
         <v>25</v>
       </c>
       <c r="Q5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="R5">
         <v>2023</v>
@@ -1406,10 +1492,10 @@
         <v>1</v>
       </c>
       <c r="B6" t="s">
-        <v>30</v>
+        <v>42</v>
       </c>
       <c r="C6" t="s">
-        <v>31</v>
+        <v>43</v>
       </c>
       <c r="D6" t="s">
         <v>20</v>
@@ -1418,25 +1504,25 @@
         <v>21</v>
       </c>
       <c r="F6" t="s">
-        <v>32</v>
+        <v>44</v>
       </c>
       <c r="G6" t="s">
+        <v>22</v>
+      </c>
+      <c r="H6" t="s">
+        <v>22</v>
+      </c>
+      <c r="I6" t="s">
+        <v>22</v>
+      </c>
+      <c r="J6" t="s">
         <v>23</v>
       </c>
-      <c r="H6" t="s">
-        <v>23</v>
-      </c>
-      <c r="I6" t="s">
-        <v>23</v>
-      </c>
-      <c r="J6" t="s">
-        <v>29</v>
-      </c>
       <c r="K6" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="L6" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="M6">
         <v>750</v>
@@ -1445,13 +1531,13 @@
         <v>24</v>
       </c>
       <c r="O6" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="P6" t="s">
         <v>25</v>
       </c>
       <c r="Q6" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="R6">
         <v>2023</v>
@@ -1462,10 +1548,10 @@
         <v>1</v>
       </c>
       <c r="B7" t="s">
-        <v>33</v>
+        <v>45</v>
       </c>
       <c r="C7" t="s">
-        <v>34</v>
+        <v>46</v>
       </c>
       <c r="D7" t="s">
         <v>20</v>
@@ -1474,25 +1560,25 @@
         <v>21</v>
       </c>
       <c r="F7" t="s">
-        <v>35</v>
+        <v>47</v>
       </c>
       <c r="G7" t="s">
+        <v>22</v>
+      </c>
+      <c r="H7" t="s">
+        <v>22</v>
+      </c>
+      <c r="I7" t="s">
+        <v>22</v>
+      </c>
+      <c r="J7" t="s">
         <v>23</v>
       </c>
-      <c r="H7" t="s">
-        <v>23</v>
-      </c>
-      <c r="I7" t="s">
-        <v>23</v>
-      </c>
-      <c r="J7" t="s">
-        <v>29</v>
-      </c>
       <c r="K7" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="L7" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="M7">
         <v>875</v>
@@ -1501,13 +1587,13 @@
         <v>24</v>
       </c>
       <c r="O7" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="P7" t="s">
         <v>25</v>
       </c>
       <c r="Q7" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="R7">
         <v>2023</v>
@@ -1518,10 +1604,10 @@
         <v>1</v>
       </c>
       <c r="B8" t="s">
-        <v>36</v>
+        <v>48</v>
       </c>
       <c r="C8" t="s">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="D8" t="s">
         <v>20</v>
@@ -1530,25 +1616,25 @@
         <v>21</v>
       </c>
       <c r="F8" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="G8" t="s">
+        <v>22</v>
+      </c>
+      <c r="H8" t="s">
+        <v>22</v>
+      </c>
+      <c r="I8" t="s">
+        <v>22</v>
+      </c>
+      <c r="J8" t="s">
         <v>23</v>
       </c>
-      <c r="H8" t="s">
-        <v>23</v>
-      </c>
-      <c r="I8" t="s">
-        <v>23</v>
-      </c>
-      <c r="J8" t="s">
-        <v>29</v>
-      </c>
       <c r="K8" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="L8" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="M8">
         <v>975</v>
@@ -1557,13 +1643,13 @@
         <v>24</v>
       </c>
       <c r="O8" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="P8" t="s">
         <v>25</v>
       </c>
       <c r="Q8" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="R8">
         <v>2023</v>
@@ -1574,10 +1660,10 @@
         <v>1</v>
       </c>
       <c r="B9" t="s">
-        <v>39</v>
+        <v>51</v>
       </c>
       <c r="C9" t="s">
-        <v>40</v>
+        <v>52</v>
       </c>
       <c r="D9" t="s">
         <v>20</v>
@@ -1586,25 +1672,25 @@
         <v>21</v>
       </c>
       <c r="F9" t="s">
-        <v>41</v>
+        <v>53</v>
       </c>
       <c r="G9" t="s">
+        <v>22</v>
+      </c>
+      <c r="H9" t="s">
+        <v>22</v>
+      </c>
+      <c r="I9" t="s">
+        <v>22</v>
+      </c>
+      <c r="J9" t="s">
         <v>23</v>
       </c>
-      <c r="H9" t="s">
-        <v>23</v>
-      </c>
-      <c r="I9" t="s">
-        <v>23</v>
-      </c>
-      <c r="J9" t="s">
-        <v>29</v>
-      </c>
       <c r="K9" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="L9" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="M9">
         <v>475</v>
@@ -1613,13 +1699,13 @@
         <v>24</v>
       </c>
       <c r="O9" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="P9" t="s">
         <v>25</v>
       </c>
       <c r="Q9" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="R9">
         <v>2023</v>
@@ -1699,37 +1785,37 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>44</v>
+        <v>30</v>
       </c>
       <c r="C2" t="s">
-        <v>45</v>
+        <v>31</v>
       </c>
       <c r="D2" t="s">
-        <v>42</v>
+        <v>28</v>
       </c>
       <c r="E2" t="s">
-        <v>43</v>
+        <v>29</v>
       </c>
       <c r="F2" t="s">
-        <v>42</v>
+        <v>28</v>
       </c>
       <c r="G2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="H2" t="s">
-        <v>42</v>
+        <v>28</v>
       </c>
       <c r="I2" t="s">
-        <v>42</v>
+        <v>28</v>
       </c>
       <c r="J2" t="s">
         <v>21</v>
       </c>
       <c r="K2" t="s">
-        <v>42</v>
+        <v>28</v>
       </c>
       <c r="L2" t="s">
-        <v>42</v>
+        <v>28</v>
       </c>
       <c r="M2">
         <v>875</v>
@@ -1738,13 +1824,13 @@
         <v>24</v>
       </c>
       <c r="O2" t="s">
-        <v>42</v>
+        <v>28</v>
       </c>
       <c r="P2" t="s">
         <v>25</v>
       </c>
       <c r="Q2" t="s">
-        <v>42</v>
+        <v>28</v>
       </c>
       <c r="R2">
         <v>2023</v>
@@ -1755,37 +1841,37 @@
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>47</v>
+        <v>33</v>
       </c>
       <c r="C3" t="s">
-        <v>48</v>
+        <v>34</v>
       </c>
       <c r="D3" t="s">
-        <v>42</v>
+        <v>28</v>
       </c>
       <c r="E3" t="s">
-        <v>43</v>
+        <v>29</v>
       </c>
       <c r="F3" t="s">
-        <v>42</v>
+        <v>28</v>
       </c>
       <c r="G3" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="H3" t="s">
-        <v>42</v>
+        <v>28</v>
       </c>
       <c r="I3" t="s">
-        <v>42</v>
+        <v>28</v>
       </c>
       <c r="J3" t="s">
         <v>21</v>
       </c>
       <c r="K3" t="s">
-        <v>42</v>
+        <v>28</v>
       </c>
       <c r="L3" t="s">
-        <v>42</v>
+        <v>28</v>
       </c>
       <c r="M3">
         <v>750</v>
@@ -1794,13 +1880,13 @@
         <v>24</v>
       </c>
       <c r="O3" t="s">
-        <v>42</v>
+        <v>28</v>
       </c>
       <c r="P3" t="s">
         <v>25</v>
       </c>
       <c r="Q3" t="s">
-        <v>42</v>
+        <v>28</v>
       </c>
       <c r="R3">
         <v>2023</v>

</xml_diff>

<commit_message>
Changing back because I'm wrong
</commit_message>
<xml_diff>
--- a/AutomateSendingOutTaxReturnsV3.xlsx
+++ b/AutomateSendingOutTaxReturnsV3.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27328"/>
   <workbookPr filterPrivacy="1" codeName="ThisWorkbook"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B767EBED-C302-48FE-9829-1C1F63DD519F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5440718-5D6C-4C98-8B70-8159329D5546}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ClientList" sheetId="1" r:id="rId1"/>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="18">
   <si>
     <t>Number</t>
   </si>
@@ -85,30 +85,6 @@
   </si>
   <si>
     <t>YearToSeal</t>
-  </si>
-  <si>
-    <t>Send Out Returns, Bill, and Efile Sigs - InvoiceInTD</t>
-  </si>
-  <si>
-    <t>none</t>
-  </si>
-  <si>
-    <t>X</t>
-  </si>
-  <si>
-    <t>Personal Tax Services - JJ</t>
-  </si>
-  <si>
-    <t>2023 1040 Return - JJ</t>
-  </si>
-  <si>
-    <t>SD3</t>
-  </si>
-  <si>
-    <t>Single, Dummy</t>
-  </si>
-  <si>
-    <t>MA-Single</t>
   </si>
 </sst>
 </file>
@@ -482,13 +458,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:R2"/>
-  <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
-  <cols>
-    <col min="14" max="14" width="14.58203125" bestFit="1" customWidth="1"/>
-  </cols>
+  <dimension ref="A1:R1"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:18" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
       <c r="B1" t="s">
         <v>1</v>
       </c>
@@ -539,68 +515,12 @@
       </c>
       <c r="R1" t="s">
         <v>17</v>
-      </c>
-    </row>
-    <row r="2" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A2">
-        <v>1</v>
-      </c>
-      <c r="B2" t="s">
-        <v>23</v>
-      </c>
-      <c r="C2" t="s">
-        <v>24</v>
-      </c>
-      <c r="D2" t="s">
-        <v>18</v>
-      </c>
-      <c r="E2" t="s">
-        <v>19</v>
-      </c>
-      <c r="F2" t="s">
-        <v>19</v>
-      </c>
-      <c r="G2" t="s">
-        <v>20</v>
-      </c>
-      <c r="H2" t="s">
-        <v>20</v>
-      </c>
-      <c r="I2" t="s">
-        <v>20</v>
-      </c>
-      <c r="J2" t="s">
-        <v>25</v>
-      </c>
-      <c r="K2" t="s">
-        <v>20</v>
-      </c>
-      <c r="L2" t="s">
-        <v>20</v>
-      </c>
-      <c r="M2">
-        <v>10</v>
-      </c>
-      <c r="N2" t="s">
-        <v>21</v>
-      </c>
-      <c r="O2" t="s">
-        <v>20</v>
-      </c>
-      <c r="P2" t="s">
-        <v>22</v>
-      </c>
-      <c r="Q2" t="s">
-        <v>20</v>
-      </c>
-      <c r="R2">
-        <v>2023</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="B1:R1" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:R1" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -608,9 +528,9 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:R1"/>
-  <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:18" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -678,9 +598,9 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:R1"/>
-  <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:18" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -747,9 +667,9 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:R1"/>
-  <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:18" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>

</xml_diff>